<commit_message>
District heating dataset update
</commit_message>
<xml_diff>
--- a/data_input/District-Heating-Dataset.xlsx
+++ b/data_input/District-Heating-Dataset.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amsuni-my.sharepoint.com/personal/f_savini_uva_nl/Documents/DECYCLE/Degrowth housing scenario project/Environmental Impact Model (Set up, Data, Results)/Current Housing State/Dominant Housing System (Income Groups, Building Types)/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6bba444eb789f06d/Documents/Internships/UVA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="196" documentId="8_{D0D2A5B3-79CC-4396-8E17-3BF5A56934ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3FA1F853-8828-4ED1-A479-045A67AF5D58}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{25D06C3D-39F4-44EA-A49B-560F679A4006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{6DC732F9-428D-4592-AB00-0563FA9F88B7}"/>
+    <workbookView xWindow="-19298" yWindow="-98" windowWidth="19396" windowHeight="10276" firstSheet="2" activeTab="2" xr2:uid="{6DC732F9-428D-4592-AB00-0563FA9F88B7}"/>
   </bookViews>
   <sheets>
     <sheet name="Municipality level" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="82">
   <si>
     <t>Municipality</t>
   </si>
@@ -371,6 +371,9 @@
   </si>
   <si>
     <t>Total (PJ)</t>
+  </si>
+  <si>
+    <t>Other</t>
   </si>
 </sst>
 </file>
@@ -2256,10 +2259,7 @@
         <v>75</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="I1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -2285,11 +2285,9 @@
         <v>0.06</v>
       </c>
       <c r="H2" s="14">
-        <v>0</v>
-      </c>
-      <c r="I2" s="15">
-        <v>5.8820000000000001E-3</v>
-      </c>
+        <v>0.04</v>
+      </c>
+      <c r="I2" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
district heating database update
</commit_message>
<xml_diff>
--- a/data_input/District-Heating-Dataset.xlsx
+++ b/data_input/District-Heating-Dataset.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6bba444eb789f06d/Documents/Internships/UVA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6bba444eb789f06d/Documents/GitHub/housing-footprints/data_input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{25D06C3D-39F4-44EA-A49B-560F679A4006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="225" documentId="8_{25D06C3D-39F4-44EA-A49B-560F679A4006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{71E1098B-D260-4042-ACE0-D1F0C3DDA44F}"/>
   <bookViews>
-    <workbookView xWindow="-19298" yWindow="-98" windowWidth="19396" windowHeight="10276" firstSheet="2" activeTab="2" xr2:uid="{6DC732F9-428D-4592-AB00-0563FA9F88B7}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10276" activeTab="2" xr2:uid="{6DC732F9-428D-4592-AB00-0563FA9F88B7}"/>
   </bookViews>
   <sheets>
     <sheet name="Municipality level" sheetId="1" r:id="rId1"/>
-    <sheet name="National average" sheetId="2" r:id="rId2"/>
-    <sheet name="National_avg_fuel" sheetId="3" r:id="rId3"/>
+    <sheet name="National average calculation" sheetId="2" r:id="rId2"/>
+    <sheet name="National average" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="83">
   <si>
     <t>Municipality</t>
   </si>
@@ -346,15 +346,9 @@
     <t xml:space="preserve"> Weighted </t>
   </si>
   <si>
-    <t>Residual heat industry</t>
-  </si>
-  <si>
     <t>Biomass power plant</t>
   </si>
   <si>
-    <t>peak gas boilers</t>
-  </si>
-  <si>
     <t>Residual heat (coal)</t>
   </si>
   <si>
@@ -367,19 +361,32 @@
     <t>Weighted</t>
   </si>
   <si>
-    <t>total weighted PJ per heat source</t>
-  </si>
-  <si>
-    <t>Total (PJ)</t>
-  </si>
-  <si>
-    <t>Other</t>
+    <t>Residual heat (industry)</t>
+  </si>
+  <si>
+    <t>Sanity Check</t>
+  </si>
+  <si>
+    <t>Total (%)</t>
+  </si>
+  <si>
+    <t>Peak gas boilers</t>
+  </si>
+  <si>
+    <t>Share</t>
+  </si>
+  <si>
+    <t>Heat_Source</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+  </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -418,7 +425,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -439,18 +446,30 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE8E8E8"/>
+        <fgColor theme="2"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
+        <fgColor theme="1" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -473,26 +492,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -505,16 +511,23 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="9" fontId="4" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="9" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="4" fillId="6" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="6" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="4" fillId="6" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -852,23 +865,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA6EB78D-E0B7-4068-9041-25EE1114C448}">
   <dimension ref="A1:H25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="35.85546875" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" customWidth="1"/>
-    <col min="3" max="3" width="19.140625" customWidth="1"/>
-    <col min="4" max="4" width="17.28515625" customWidth="1"/>
-    <col min="5" max="5" width="18.85546875" customWidth="1"/>
-    <col min="6" max="6" width="56.5703125" customWidth="1"/>
-    <col min="7" max="7" width="29.140625" customWidth="1"/>
+    <col min="1" max="1" width="35.86328125" customWidth="1"/>
+    <col min="2" max="2" width="23.73046875" customWidth="1"/>
+    <col min="3" max="3" width="19.1328125" customWidth="1"/>
+    <col min="4" max="4" width="17.265625" customWidth="1"/>
+    <col min="5" max="5" width="18.86328125" customWidth="1"/>
+    <col min="6" max="6" width="56.59765625" customWidth="1"/>
+    <col min="7" max="7" width="29.1328125" customWidth="1"/>
     <col min="8" max="8" width="29" customWidth="1"/>
-    <col min="9" max="9" width="15.5703125" customWidth="1"/>
-    <col min="10" max="10" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="12.42578125" customWidth="1"/>
-    <col min="12" max="12" width="12.140625" customWidth="1"/>
+    <col min="9" max="9" width="15.59765625" customWidth="1"/>
+    <col min="10" max="10" width="11.86328125" customWidth="1"/>
+    <col min="11" max="11" width="12.3984375" customWidth="1"/>
+    <col min="12" max="12" width="12.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -891,7 +904,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -914,7 +927,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -940,7 +953,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -963,7 +976,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -986,7 +999,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -1009,7 +1022,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -1035,7 +1048,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>24</v>
       </c>
@@ -1058,7 +1071,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>28</v>
       </c>
@@ -1081,7 +1094,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>31</v>
       </c>
@@ -1104,7 +1117,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>33</v>
       </c>
@@ -1127,7 +1140,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>35</v>
       </c>
@@ -1150,7 +1163,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>37</v>
       </c>
@@ -1173,7 +1186,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>39</v>
       </c>
@@ -1196,7 +1209,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>43</v>
       </c>
@@ -1219,7 +1232,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>45</v>
       </c>
@@ -1242,7 +1255,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>47</v>
       </c>
@@ -1265,7 +1278,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>49</v>
       </c>
@@ -1286,7 +1299,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>51</v>
       </c>
@@ -1307,7 +1320,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>53</v>
       </c>
@@ -1327,7 +1340,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>55</v>
       </c>
@@ -1350,7 +1363,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>59</v>
       </c>
@@ -1373,7 +1386,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>63</v>
       </c>
@@ -1393,7 +1406,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>65</v>
       </c>
@@ -1413,7 +1426,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>67</v>
       </c>
@@ -1478,750 +1491,935 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00BCDC15-0AA9-4C30-AC95-68925AD22B21}">
-  <dimension ref="A1:R22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:S22"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
+    <col min="19" max="19" width="12.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="7" t="s">
         <v>68</v>
       </c>
       <c r="D1" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="7" t="s">
         <v>70</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="G1" s="8" t="s">
-        <v>72</v>
+      <c r="G1" s="7" t="s">
+        <v>77</v>
       </c>
       <c r="H1" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="I1" s="8" t="s">
-        <v>73</v>
+      <c r="I1" s="7" t="s">
+        <v>72</v>
       </c>
       <c r="J1" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="K1" s="8" t="s">
-        <v>74</v>
+      <c r="K1" s="7" t="s">
+        <v>80</v>
       </c>
       <c r="L1" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="M1" s="8" t="s">
-        <v>75</v>
+      <c r="M1" s="7" t="s">
+        <v>73</v>
       </c>
       <c r="N1" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="O1" s="8" t="s">
-        <v>76</v>
+      <c r="O1" s="7" t="s">
+        <v>74</v>
       </c>
       <c r="P1" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="Q1" t="s">
-        <v>77</v>
-      </c>
-      <c r="R1" t="s">
+      <c r="Q1" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="R1" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="S1" s="2" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="8">
+      <c r="B2" s="7">
         <v>2.9</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="11">
         <v>0.72</v>
       </c>
       <c r="D2" s="8">
-        <v>2.09</v>
-      </c>
-      <c r="E2" s="8"/>
+        <f t="shared" ref="D2:D7" si="0">C2*B2</f>
+        <v>2.0880000000000001</v>
+      </c>
+      <c r="E2" s="7"/>
       <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
+      <c r="G2" s="7"/>
       <c r="H2" s="8"/>
-      <c r="I2" s="9">
+      <c r="I2" s="11">
         <v>0.1</v>
       </c>
-      <c r="J2" s="8">
+      <c r="J2" s="15">
+        <f>I2*B2</f>
         <v>0.28999999999999998</v>
       </c>
-      <c r="K2" s="8"/>
-      <c r="L2" s="8"/>
-      <c r="M2" s="8"/>
+      <c r="K2" s="11">
+        <v>0.18</v>
+      </c>
+      <c r="L2" s="8">
+        <f t="shared" ref="L2:L7" si="1">K2*B2</f>
+        <v>0.52200000000000002</v>
+      </c>
+      <c r="M2" s="7"/>
       <c r="N2" s="8"/>
-      <c r="O2" s="8"/>
+      <c r="O2" s="7"/>
       <c r="P2" s="8"/>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="Q2" s="2"/>
+      <c r="R2" s="9"/>
+      <c r="S2" s="12">
+        <f>SUM(C2,I2,K2)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A3" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="7">
         <v>3.4</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="11">
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="D3" s="8">
-        <v>0.24</v>
-      </c>
-      <c r="E3" s="9">
+        <f t="shared" si="0"/>
+        <v>0.23800000000000002</v>
+      </c>
+      <c r="E3" s="11">
         <v>0.54</v>
       </c>
       <c r="F3" s="8">
-        <v>1.84</v>
-      </c>
-      <c r="G3" s="9">
+        <f>E3*B3</f>
+        <v>1.8360000000000001</v>
+      </c>
+      <c r="G3" s="11">
         <v>0.18</v>
       </c>
       <c r="H3" s="8">
-        <v>0.61</v>
-      </c>
-      <c r="I3" s="9">
+        <f>G3*B3</f>
+        <v>0.61199999999999999</v>
+      </c>
+      <c r="I3" s="11">
         <v>0.15</v>
       </c>
-      <c r="J3" s="8">
+      <c r="J3" s="15">
+        <f>I3*B3</f>
         <v>0.51</v>
       </c>
-      <c r="K3" s="9">
+      <c r="K3" s="11">
         <v>0.06</v>
       </c>
       <c r="L3" s="8">
+        <f t="shared" si="1"/>
+        <v>0.20399999999999999</v>
+      </c>
+      <c r="M3" s="7"/>
+      <c r="N3" s="8"/>
+      <c r="O3" s="7"/>
+      <c r="P3" s="8"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="9"/>
+      <c r="S3" s="12">
+        <f>SUM(C3,E3,G3,I3,K3)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A4" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="7">
+        <v>1.6</v>
+      </c>
+      <c r="C4" s="11">
+        <v>0.6</v>
+      </c>
+      <c r="D4" s="15">
+        <f t="shared" si="0"/>
+        <v>0.96</v>
+      </c>
+      <c r="E4" s="11">
+        <v>0.16</v>
+      </c>
+      <c r="F4" s="8">
+        <f>E4*B4</f>
+        <v>0.25600000000000001</v>
+      </c>
+      <c r="G4" s="7"/>
+      <c r="H4" s="8"/>
+      <c r="I4" s="11">
+        <v>0.21</v>
+      </c>
+      <c r="J4" s="8">
+        <f>I4*B4</f>
+        <v>0.33600000000000002</v>
+      </c>
+      <c r="K4" s="11">
+        <v>0.03</v>
+      </c>
+      <c r="L4" s="8">
+        <f t="shared" si="1"/>
+        <v>4.8000000000000001E-2</v>
+      </c>
+      <c r="M4" s="7"/>
+      <c r="N4" s="8"/>
+      <c r="O4" s="7"/>
+      <c r="P4" s="8"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="9"/>
+      <c r="S4" s="12">
+        <f>SUM(C4,E4,I4,K4)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A5" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="7">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C5" s="11">
+        <v>0.49</v>
+      </c>
+      <c r="D5" s="8">
+        <f t="shared" si="0"/>
+        <v>0.53900000000000003</v>
+      </c>
+      <c r="E5" s="7"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="11">
+        <v>0.21</v>
+      </c>
+      <c r="H5" s="8">
+        <f>G5*B5</f>
+        <v>0.23100000000000001</v>
+      </c>
+      <c r="I5" s="7"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="11">
+        <v>0.3</v>
+      </c>
+      <c r="L5" s="15">
+        <f t="shared" si="1"/>
+        <v>0.33</v>
+      </c>
+      <c r="M5" s="7"/>
+      <c r="N5" s="8"/>
+      <c r="O5" s="7"/>
+      <c r="P5" s="8"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="9"/>
+      <c r="S5" s="12">
+        <f>SUM(C5,G5,K5)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A6" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="C6" s="11">
+        <v>0.62</v>
+      </c>
+      <c r="D6" s="8">
+        <f t="shared" si="0"/>
+        <v>0.186</v>
+      </c>
+      <c r="E6" s="7"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="11">
+        <v>0.01</v>
+      </c>
+      <c r="H6" s="8">
+        <f>G6*B6</f>
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="I6" s="7"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="11">
+        <v>0.37</v>
+      </c>
+      <c r="L6" s="8">
+        <f t="shared" si="1"/>
+        <v>0.111</v>
+      </c>
+      <c r="M6" s="7"/>
+      <c r="N6" s="8"/>
+      <c r="O6" s="7"/>
+      <c r="P6" s="8"/>
+      <c r="Q6" s="2"/>
+      <c r="R6" s="9"/>
+      <c r="S6" s="12">
+        <f>SUM(C6,G6,K6)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A7" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="7">
+        <v>1.8</v>
+      </c>
+      <c r="C7" s="11">
+        <v>0.74</v>
+      </c>
+      <c r="D7" s="8">
+        <f t="shared" si="0"/>
+        <v>1.3320000000000001</v>
+      </c>
+      <c r="E7" s="7"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="11">
+        <v>0.03</v>
+      </c>
+      <c r="H7" s="8">
+        <f>G7*B7</f>
+        <v>5.3999999999999999E-2</v>
+      </c>
+      <c r="I7" s="7"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="11">
+        <v>0.23</v>
+      </c>
+      <c r="L7" s="8">
+        <f t="shared" si="1"/>
+        <v>0.41400000000000003</v>
+      </c>
+      <c r="M7" s="7"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="7"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="9"/>
+      <c r="S7" s="12">
+        <f>SUM(C7,G7,K7)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A8" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="7">
+        <v>1</v>
+      </c>
+      <c r="C8" s="7"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="11">
+        <v>1</v>
+      </c>
+      <c r="F8" s="8">
+        <f>E8*B8</f>
+        <v>1</v>
+      </c>
+      <c r="G8" s="7"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="7"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="2"/>
+      <c r="R8" s="9"/>
+      <c r="S8" s="12">
+        <f>SUM(E8)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A9" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="7">
+        <v>1.9</v>
+      </c>
+      <c r="C9" s="11">
+        <v>0.93</v>
+      </c>
+      <c r="D9" s="8">
+        <f>C9*B9</f>
+        <v>1.7669999999999999</v>
+      </c>
+      <c r="E9" s="7"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="11">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="L9" s="8">
+        <f>K9*B9</f>
+        <v>0.13300000000000001</v>
+      </c>
+      <c r="M9" s="7"/>
+      <c r="N9" s="8"/>
+      <c r="O9" s="7"/>
+      <c r="P9" s="8"/>
+      <c r="Q9" s="2"/>
+      <c r="R9" s="9"/>
+      <c r="S9" s="12">
+        <f>SUM(C9,K9)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A10" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="7">
         <v>0.2</v>
       </c>
-      <c r="M3" s="8"/>
-      <c r="N3" s="8"/>
-      <c r="O3" s="8"/>
-      <c r="P3" s="8"/>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="8">
-        <v>1.6</v>
-      </c>
-      <c r="C4" s="9">
-        <v>0.6</v>
-      </c>
-      <c r="D4" s="8">
+      <c r="C10" s="11">
+        <v>0.11</v>
+      </c>
+      <c r="D10" s="8">
+        <f>C10*B10</f>
+        <v>2.2000000000000002E-2</v>
+      </c>
+      <c r="E10" s="7"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="11">
+        <v>0.46</v>
+      </c>
+      <c r="J10" s="8">
+        <f>I10*B10</f>
+        <v>9.2000000000000012E-2</v>
+      </c>
+      <c r="K10" s="11">
+        <v>0.43</v>
+      </c>
+      <c r="L10" s="8">
+        <f>K10*B10</f>
+        <v>8.6000000000000007E-2</v>
+      </c>
+      <c r="M10" s="7"/>
+      <c r="N10" s="8"/>
+      <c r="O10" s="7"/>
+      <c r="P10" s="8"/>
+      <c r="Q10" s="2"/>
+      <c r="R10" s="9"/>
+      <c r="S10" s="12">
+        <f>SUM(C10,I10,K10)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A11" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="7">
+        <v>0.7</v>
+      </c>
+      <c r="C11" s="11">
+        <v>0.72</v>
+      </c>
+      <c r="D11" s="8">
+        <f>C11*B11</f>
+        <v>0.504</v>
+      </c>
+      <c r="E11" s="7"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="11">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="L11" s="8">
+        <f>K11*B11</f>
+        <v>0.19600000000000001</v>
+      </c>
+      <c r="M11" s="7"/>
+      <c r="N11" s="8"/>
+      <c r="O11" s="7"/>
+      <c r="P11" s="8"/>
+      <c r="Q11" s="2"/>
+      <c r="R11" s="9"/>
+      <c r="S11" s="12">
+        <f>SUM(C11,K11)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A12" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="7">
+        <v>0.7</v>
+      </c>
+      <c r="C12" s="7"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="11">
         <v>0.96</v>
       </c>
-      <c r="E4" s="9">
-        <v>0.16</v>
-      </c>
-      <c r="F4" s="8">
-        <v>0.26</v>
-      </c>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="9">
-        <v>0.21</v>
-      </c>
-      <c r="J4" s="8">
-        <v>0.34</v>
-      </c>
-      <c r="K4" s="9">
-        <v>0.03</v>
-      </c>
-      <c r="L4" s="8">
+      <c r="F12" s="8">
+        <f>E12*B12</f>
+        <v>0.67199999999999993</v>
+      </c>
+      <c r="G12" s="7"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="11">
+        <v>0.04</v>
+      </c>
+      <c r="L12" s="8">
+        <f>K12*B12</f>
+        <v>2.7999999999999997E-2</v>
+      </c>
+      <c r="M12" s="7"/>
+      <c r="N12" s="8"/>
+      <c r="O12" s="7"/>
+      <c r="P12" s="8"/>
+      <c r="Q12" s="2"/>
+      <c r="R12" s="9"/>
+      <c r="S12" s="12">
+        <f>SUM(E12,K12)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A13" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="C13" s="7"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="11">
+        <v>0.95</v>
+      </c>
+      <c r="F13" s="15">
+        <f>E13*B13</f>
+        <v>0.19</v>
+      </c>
+      <c r="G13" s="7"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="11">
         <v>0.05</v>
       </c>
-      <c r="M4" s="8"/>
-      <c r="N4" s="8"/>
-      <c r="O4" s="8"/>
-      <c r="P4" s="8"/>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="8">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="C5" s="9">
-        <v>0.49</v>
-      </c>
-      <c r="D5" s="8">
-        <v>0.54</v>
-      </c>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="9">
-        <v>0.21</v>
-      </c>
-      <c r="H5" s="8">
-        <v>0.23</v>
-      </c>
-      <c r="I5" s="8"/>
-      <c r="J5" s="8"/>
-      <c r="K5" s="9">
-        <v>0.3</v>
-      </c>
-      <c r="L5" s="8">
-        <v>0.33</v>
-      </c>
-      <c r="M5" s="8"/>
-      <c r="N5" s="8"/>
-      <c r="O5" s="8"/>
-      <c r="P5" s="8"/>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="8">
-        <v>0.3</v>
-      </c>
-      <c r="C6" s="9">
-        <v>0.62</v>
-      </c>
-      <c r="D6" s="8">
-        <v>0.19</v>
-      </c>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="9">
-        <v>0.01</v>
-      </c>
-      <c r="H6" s="8">
-        <v>0</v>
-      </c>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
-      <c r="K6" s="9">
-        <v>0.37</v>
-      </c>
-      <c r="L6" s="8">
+      <c r="L13" s="15">
+        <f>K13*B13</f>
+        <v>1.0000000000000002E-2</v>
+      </c>
+      <c r="M13" s="7"/>
+      <c r="N13" s="8"/>
+      <c r="O13" s="7"/>
+      <c r="P13" s="8"/>
+      <c r="Q13" s="2"/>
+      <c r="R13" s="9"/>
+      <c r="S13" s="12">
+        <f>SUM(E13,K13)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A14" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" s="7">
+        <v>2.4</v>
+      </c>
+      <c r="C14" s="11">
         <v>0.11</v>
       </c>
-      <c r="M6" s="8"/>
-      <c r="N6" s="8"/>
-      <c r="O6" s="8"/>
-      <c r="P6" s="8"/>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7" s="8">
-        <v>1.8</v>
-      </c>
-      <c r="C7" s="9">
-        <v>0.74</v>
-      </c>
-      <c r="D7" s="8">
-        <v>1.33</v>
-      </c>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="9">
-        <v>0.03</v>
-      </c>
-      <c r="H7" s="8">
-        <v>0.05</v>
-      </c>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="9">
-        <v>0.23</v>
-      </c>
-      <c r="L7" s="8">
-        <v>0.41</v>
-      </c>
-      <c r="M7" s="8"/>
-      <c r="N7" s="8"/>
-      <c r="O7" s="8"/>
-      <c r="P7" s="8"/>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="B8" s="8">
-        <v>1</v>
-      </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="9">
-        <v>1</v>
-      </c>
-      <c r="F8" s="8">
-        <v>1</v>
-      </c>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="8"/>
-      <c r="L8" s="8"/>
-      <c r="M8" s="8"/>
-      <c r="N8" s="8"/>
-      <c r="O8" s="8"/>
-      <c r="P8" s="8"/>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="B9" s="8">
-        <v>1.9</v>
-      </c>
-      <c r="C9" s="9">
-        <v>0.93</v>
-      </c>
-      <c r="D9" s="8">
-        <v>1.77</v>
-      </c>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
-      <c r="K9" s="9">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="L9" s="8">
-        <v>0.13</v>
-      </c>
-      <c r="M9" s="8"/>
-      <c r="N9" s="8"/>
-      <c r="O9" s="8"/>
-      <c r="P9" s="8"/>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" s="8">
-        <v>0.2</v>
-      </c>
-      <c r="C10" s="9">
-        <v>0.11</v>
-      </c>
-      <c r="D10" s="8">
-        <v>0.02</v>
-      </c>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="9">
-        <v>0.46</v>
-      </c>
-      <c r="J10" s="8">
-        <v>0.09</v>
-      </c>
-      <c r="K10" s="9">
-        <v>0.43</v>
-      </c>
-      <c r="L10" s="8">
-        <v>0.09</v>
-      </c>
-      <c r="M10" s="8"/>
-      <c r="N10" s="8"/>
-      <c r="O10" s="8"/>
-      <c r="P10" s="8"/>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="B11" s="8">
-        <v>0.7</v>
-      </c>
-      <c r="C11" s="9">
-        <v>0.72</v>
-      </c>
-      <c r="D11" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
-      <c r="J11" s="8"/>
-      <c r="K11" s="9">
-        <v>0.28000000000000003</v>
-      </c>
-      <c r="L11" s="8">
-        <v>0.2</v>
-      </c>
-      <c r="M11" s="8"/>
-      <c r="N11" s="8"/>
-      <c r="O11" s="8"/>
-      <c r="P11" s="8"/>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="B12" s="8">
-        <v>0.7</v>
-      </c>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="9">
-        <v>0.96</v>
-      </c>
-      <c r="F12" s="8">
-        <v>0.67</v>
-      </c>
-      <c r="G12" s="8"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
-      <c r="K12" s="9">
-        <v>0.04</v>
-      </c>
-      <c r="L12" s="8">
-        <v>0.03</v>
-      </c>
-      <c r="M12" s="8"/>
-      <c r="N12" s="8"/>
-      <c r="O12" s="8"/>
-      <c r="P12" s="8"/>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A13" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="B13" s="8">
-        <v>0.2</v>
-      </c>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="9">
-        <v>0.95</v>
-      </c>
-      <c r="F13" s="8">
-        <v>0.19</v>
-      </c>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
-      <c r="J13" s="8"/>
-      <c r="K13" s="9">
-        <v>0.05</v>
-      </c>
-      <c r="L13" s="8">
-        <v>0.01</v>
-      </c>
-      <c r="M13" s="8"/>
-      <c r="N13" s="8"/>
-      <c r="O13" s="8"/>
-      <c r="P13" s="8"/>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A14" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B14" s="8">
-        <v>2.4</v>
-      </c>
-      <c r="C14" s="9">
-        <v>0.11</v>
-      </c>
       <c r="D14" s="8">
-        <v>0.34</v>
-      </c>
-      <c r="E14" s="8"/>
+        <f>C14*B14</f>
+        <v>0.26400000000000001</v>
+      </c>
+      <c r="E14" s="7"/>
       <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
+      <c r="G14" s="7"/>
       <c r="H14" s="8"/>
-      <c r="I14" s="9">
+      <c r="I14" s="11">
         <v>0.31</v>
       </c>
       <c r="J14" s="8">
-        <v>0.79</v>
-      </c>
-      <c r="K14" s="8"/>
+        <f>I14*B14</f>
+        <v>0.74399999999999999</v>
+      </c>
+      <c r="K14" s="7"/>
       <c r="L14" s="8"/>
-      <c r="M14" s="9">
+      <c r="M14" s="11">
         <v>0.53</v>
       </c>
       <c r="N14" s="8">
-        <v>1.27</v>
-      </c>
-      <c r="O14" s="8"/>
+        <f>M14*B14</f>
+        <v>1.272</v>
+      </c>
+      <c r="O14" s="7"/>
       <c r="P14" s="8"/>
       <c r="Q14" s="12">
         <v>0.05</v>
       </c>
-      <c r="R14">
+      <c r="R14" s="16">
         <f>Q14*B14</f>
         <v>0.12</v>
       </c>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A15" s="8" t="s">
+      <c r="S14" s="12">
+        <f>SUM(C14,I14,M14,Q14)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A15" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B15" s="8">
+      <c r="B15" s="7">
         <v>0.5</v>
       </c>
-      <c r="C15" s="8"/>
+      <c r="C15" s="7"/>
       <c r="D15" s="8"/>
-      <c r="E15" s="9">
+      <c r="E15" s="11">
         <v>0.24</v>
       </c>
-      <c r="F15" s="8">
+      <c r="F15" s="15">
+        <f>E15*B15</f>
         <v>0.12</v>
       </c>
-      <c r="G15" s="8"/>
+      <c r="G15" s="7"/>
       <c r="H15" s="8"/>
-      <c r="I15" s="9">
+      <c r="I15" s="11">
         <v>0.72</v>
       </c>
-      <c r="J15" s="8">
+      <c r="J15" s="15">
+        <f>I15*B15</f>
         <v>0.36</v>
       </c>
-      <c r="K15" s="8"/>
+      <c r="K15" s="7"/>
       <c r="L15" s="8"/>
-      <c r="M15" s="8"/>
+      <c r="M15" s="7"/>
       <c r="N15" s="8"/>
-      <c r="O15" s="9">
+      <c r="O15" s="11">
         <v>0.04</v>
       </c>
-      <c r="P15" s="8">
+      <c r="P15" s="15">
+        <f>O15*B15</f>
         <v>0.02</v>
       </c>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
+      <c r="Q15" s="2"/>
+      <c r="R15" s="9"/>
+      <c r="S15" s="12">
+        <f>SUM(E15,I15,O15)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="8">
+      <c r="B16" s="7">
         <v>0.3</v>
       </c>
-      <c r="C16" s="9">
+      <c r="C16" s="11">
         <v>1</v>
       </c>
-      <c r="D16" s="8">
+      <c r="D16" s="15">
+        <f>C16*B16</f>
         <v>0.3</v>
       </c>
-      <c r="E16" s="8"/>
+      <c r="E16" s="7"/>
       <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
+      <c r="G16" s="7"/>
       <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
+      <c r="I16" s="7"/>
       <c r="J16" s="8"/>
-      <c r="K16" s="8"/>
+      <c r="K16" s="7"/>
       <c r="L16" s="8"/>
-      <c r="M16" s="8"/>
+      <c r="M16" s="7"/>
       <c r="N16" s="8"/>
-      <c r="O16" s="8"/>
+      <c r="O16" s="7"/>
       <c r="P16" s="8"/>
-    </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A17" s="8" t="s">
+      <c r="Q16" s="2"/>
+      <c r="R16" s="9"/>
+      <c r="S16" s="12">
+        <f>SUM(C16)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A17" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B17" s="8">
+      <c r="B17" s="7">
         <v>0.2</v>
       </c>
-      <c r="C17" s="9">
+      <c r="C17" s="11">
         <v>0.5</v>
       </c>
-      <c r="D17" s="8">
+      <c r="D17" s="15">
+        <f>C17*B17</f>
         <v>0.1</v>
       </c>
-      <c r="E17" s="8"/>
+      <c r="E17" s="7"/>
       <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
+      <c r="G17" s="7"/>
       <c r="H17" s="8"/>
-      <c r="I17" s="9">
+      <c r="I17" s="11">
         <v>0.5</v>
       </c>
-      <c r="J17" s="8">
+      <c r="J17" s="15">
+        <f>I17*B17</f>
         <v>0.1</v>
       </c>
-      <c r="K17" s="8"/>
+      <c r="K17" s="7"/>
       <c r="L17" s="8"/>
-      <c r="M17" s="8"/>
+      <c r="M17" s="7"/>
       <c r="N17" s="8"/>
-      <c r="O17" s="8"/>
+      <c r="O17" s="7"/>
       <c r="P17" s="8"/>
-    </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
+      <c r="Q17" s="2"/>
+      <c r="R17" s="9"/>
+      <c r="S17" s="12">
+        <f>SUM(C17,I17)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A18" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B18" s="7">
         <v>0.4</v>
       </c>
-      <c r="C18" s="8"/>
+      <c r="C18" s="7"/>
       <c r="D18" s="8"/>
-      <c r="E18" s="9">
+      <c r="E18" s="11">
         <v>0.19</v>
       </c>
       <c r="F18" s="8">
-        <v>0.08</v>
-      </c>
-      <c r="G18" s="8"/>
+        <f>E18*B18</f>
+        <v>7.6000000000000012E-2</v>
+      </c>
+      <c r="G18" s="7"/>
       <c r="H18" s="8"/>
-      <c r="I18" s="9">
+      <c r="I18" s="11">
         <v>0.79</v>
       </c>
       <c r="J18" s="8">
-        <v>0.32</v>
-      </c>
-      <c r="K18" s="9">
+        <f>I18*B18</f>
+        <v>0.31600000000000006</v>
+      </c>
+      <c r="K18" s="11">
         <v>0.02</v>
       </c>
       <c r="L18" s="8">
-        <v>0.01</v>
-      </c>
-      <c r="M18" s="8"/>
+        <f>K18*B18</f>
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="M18" s="7"/>
       <c r="N18" s="8"/>
-      <c r="O18" s="8"/>
+      <c r="O18" s="7"/>
       <c r="P18" s="8"/>
-    </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A19" s="8" t="s">
+      <c r="Q18" s="2"/>
+      <c r="R18" s="9"/>
+      <c r="S18" s="12">
+        <f>SUM(E18,I18,K18)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A19" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="B19" s="8">
+      <c r="B19" s="7">
         <v>0.8</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="11">
         <v>0.34</v>
       </c>
       <c r="D19" s="8">
-        <v>0.27</v>
-      </c>
-      <c r="E19" s="8"/>
+        <f>C19*B19</f>
+        <v>0.27200000000000002</v>
+      </c>
+      <c r="E19" s="7"/>
       <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
+      <c r="G19" s="7"/>
       <c r="H19" s="8"/>
-      <c r="I19" s="9">
+      <c r="I19" s="11">
         <v>0.66</v>
       </c>
       <c r="J19" s="8">
-        <v>0.53</v>
-      </c>
-      <c r="K19" s="8"/>
+        <f>I19*B19</f>
+        <v>0.52800000000000002</v>
+      </c>
+      <c r="K19" s="7"/>
       <c r="L19" s="8"/>
-      <c r="M19" s="8"/>
+      <c r="M19" s="7"/>
       <c r="N19" s="8"/>
-      <c r="O19" s="8"/>
+      <c r="O19" s="7"/>
       <c r="P19" s="8"/>
-    </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A20" s="8" t="s">
+      <c r="Q19" s="2"/>
+      <c r="R19" s="9"/>
+      <c r="S19" s="12">
+        <f>SUM(C19,I19)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A20" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="13">
+        <f>SUM(B2:B19)</f>
         <v>20.399999999999999</v>
       </c>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8">
-        <v>8.64</v>
-      </c>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8">
-        <v>4.1500000000000004</v>
-      </c>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8">
+      <c r="C20" s="13"/>
+      <c r="D20" s="13">
+        <f>SUM(D2:D19)</f>
+        <v>8.5719999999999992</v>
+      </c>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13">
+        <f>SUM(F2:F19)</f>
+        <v>4.1499999999999995</v>
+      </c>
+      <c r="G20" s="13"/>
+      <c r="H20" s="13">
+        <f>SUM(H2:H19)</f>
         <v>0.9</v>
       </c>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8">
-        <v>3.32</v>
-      </c>
-      <c r="K20" s="8"/>
-      <c r="L20" s="8">
-        <v>1.57</v>
-      </c>
-      <c r="M20" s="8"/>
-      <c r="N20" s="8">
-        <v>1.27</v>
-      </c>
-      <c r="O20" s="8"/>
-      <c r="P20" s="8">
+      <c r="I20" s="13"/>
+      <c r="J20" s="13">
+        <f>SUM(J2:J19)</f>
+        <v>3.2760000000000002</v>
+      </c>
+      <c r="K20" s="13"/>
+      <c r="L20" s="13">
+        <f>SUM(L2:L19)</f>
+        <v>2.09</v>
+      </c>
+      <c r="M20" s="13"/>
+      <c r="N20" s="13">
+        <f>SUM(N2:N19)</f>
+        <v>1.272</v>
+      </c>
+      <c r="O20" s="13"/>
+      <c r="P20" s="13">
+        <f>SUM(P2:P19)</f>
         <v>0.02</v>
       </c>
-      <c r="R20">
-        <f>SUM(R14)</f>
+      <c r="Q20" s="14"/>
+      <c r="R20" s="14">
+        <f>SUM(R2:R19)</f>
         <v>0.12</v>
       </c>
-    </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A21" s="8"/>
-      <c r="B21" s="8"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="8"/>
-      <c r="I21" s="8"/>
-      <c r="J21" s="8"/>
-      <c r="K21" s="8"/>
-      <c r="L21" s="8"/>
-      <c r="M21" s="8"/>
-      <c r="N21" s="8"/>
-      <c r="O21" s="8"/>
-      <c r="P21" s="8"/>
-    </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A22" s="8" t="s">
+      <c r="S20" s="14">
+        <f>SUM(C20:R20)</f>
+        <v>20.399999999999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A21" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="11">
-        <v>0.42</v>
-      </c>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11">
-        <v>0.2</v>
-      </c>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11">
-        <v>0.04</v>
-      </c>
-      <c r="I22" s="11"/>
-      <c r="J22" s="11">
-        <v>0.16</v>
-      </c>
-      <c r="K22" s="11"/>
-      <c r="L22" s="11">
-        <v>0.08</v>
-      </c>
-      <c r="M22" s="11"/>
-      <c r="N22" s="11">
-        <v>0.06</v>
-      </c>
-      <c r="O22" s="8"/>
-      <c r="P22" s="8">
-        <v>0</v>
-      </c>
-      <c r="R22">
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17">
+        <f>D20/B20</f>
+        <v>0.42019607843137252</v>
+      </c>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17">
+        <f>F20/B20</f>
+        <v>0.20343137254901961</v>
+      </c>
+      <c r="G21" s="17"/>
+      <c r="H21" s="17">
+        <f>H20/B20</f>
+        <v>4.4117647058823532E-2</v>
+      </c>
+      <c r="I21" s="17"/>
+      <c r="J21" s="17">
+        <f>J20/B20</f>
+        <v>0.16058823529411767</v>
+      </c>
+      <c r="K21" s="17"/>
+      <c r="L21" s="17">
+        <f>L20/B20</f>
+        <v>0.10245098039215686</v>
+      </c>
+      <c r="M21" s="17"/>
+      <c r="N21" s="17">
+        <f>N20/B20</f>
+        <v>6.235294117647059E-2</v>
+      </c>
+      <c r="O21" s="17"/>
+      <c r="P21" s="19">
+        <f>P20/B20</f>
+        <v>9.8039215686274508E-4</v>
+      </c>
+      <c r="Q21" s="18"/>
+      <c r="R21" s="18">
         <f>R20/B20</f>
         <v>5.8823529411764705E-3</v>
       </c>
+      <c r="S21" s="18">
+        <f>SUM(D21:R21)</f>
+        <v>0.99999999999999989</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="B22" s="6"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
+      <c r="G22" s="6"/>
+      <c r="H22" s="6"/>
+      <c r="I22" s="6"/>
+      <c r="J22" s="6"/>
+      <c r="K22" s="6"/>
+      <c r="L22" s="6"/>
+      <c r="M22" s="6"/>
+      <c r="N22" s="6"/>
+      <c r="O22" s="6"/>
+      <c r="P22" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2229,65 +2427,89 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73FB08EA-F0C7-473D-BCE0-87644B6D0EAA}">
-  <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="8" max="8" width="9.28515625" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBFA3CA6-DEFB-43EB-809E-2546365F8FF1}">
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A1" s="22" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="22" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A2" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2" s="20">
+        <f>'National average calculation'!D21</f>
+        <v>0.42019607843137252</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A3" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B3" s="20">
+        <f>'National average calculation'!F21</f>
+        <v>0.20343137254901961</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A4" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B4" s="20">
+        <f>'National average calculation'!H21</f>
+        <v>4.4117647058823532E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A5" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="B5" s="20">
+        <f>'National average calculation'!J21</f>
+        <v>0.16058823529411767</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A6" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B1" t="s">
-        <v>68</v>
-      </c>
-      <c r="C1" t="s">
-        <v>70</v>
-      </c>
-      <c r="D1" t="s">
-        <v>72</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="B6" s="20">
+        <f>'National average calculation'!L21</f>
+        <v>0.10245098039215686</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A7" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="F1" t="s">
+      <c r="B7" s="20">
+        <f>'National average calculation'!N21</f>
+        <v>6.235294117647059E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A8" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="G1" t="s">
+      <c r="B8" s="21">
+        <f>'National average calculation'!P21</f>
+        <v>9.8039215686274508E-4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A9" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="H1" s="8" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>20.399999999999999</v>
-      </c>
-      <c r="B2" s="13">
-        <v>0.42</v>
-      </c>
-      <c r="C2" s="13">
-        <v>0.2</v>
-      </c>
-      <c r="D2" s="13">
-        <v>0.04</v>
-      </c>
-      <c r="E2" s="13">
-        <v>0.16</v>
-      </c>
-      <c r="F2" s="13">
-        <v>0.08</v>
-      </c>
-      <c r="G2" s="13">
-        <v>0.06</v>
-      </c>
-      <c r="H2" s="14">
-        <v>0.04</v>
-      </c>
-      <c r="I2" s="15"/>
+      <c r="B9" s="20">
+        <f>'National average calculation'!R21</f>
+        <v>5.8823529411764705E-3</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
adjusted district heating to verhagen
</commit_message>
<xml_diff>
--- a/data_input/District-Heating-Dataset.xlsx
+++ b/data_input/District-Heating-Dataset.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6bba444eb789f06d/Documents/GitHub/housing-footprints/data_input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Mira/Documents/IE/REAL UTOPIAN HOUSING/Post-GrowthHousingScenarios/Code/housing-footprints/data_input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="225" documentId="8_{25D06C3D-39F4-44EA-A49B-560F679A4006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{71E1098B-D260-4042-ACE0-D1F0C3DDA44F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2459861B-5ABE-CF4F-86D4-F596B0044739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10276" activeTab="2" xr2:uid="{6DC732F9-428D-4592-AB00-0563FA9F88B7}"/>
+    <workbookView xWindow="36540" yWindow="1340" windowWidth="27980" windowHeight="13700" activeTab="2" xr2:uid="{6DC732F9-428D-4592-AB00-0563FA9F88B7}"/>
   </bookViews>
   <sheets>
     <sheet name="Municipality level" sheetId="1" r:id="rId1"/>
     <sheet name="National average calculation" sheetId="2" r:id="rId2"/>
     <sheet name="National average" sheetId="3" r:id="rId3"/>
+    <sheet name="GHG intensity" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="104">
   <si>
     <t>Municipality</t>
   </si>
@@ -378,6 +379,129 @@
   <si>
     <t>Heat_Source</t>
   </si>
+  <si>
+    <t>(a)</t>
+  </si>
+  <si>
+    <t>Energy source</t>
+  </si>
+  <si>
+    <r>
+      <t>Gram CO</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>/GJ</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Gram CO</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>/kWh heat</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>CO</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> intensity (natural gas = 1)</t>
+    </r>
+  </si>
+  <si>
+    <t>Temperature</t>
+  </si>
+  <si>
+    <t>Natural gas</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Biomass</t>
+  </si>
+  <si>
+    <t>LT</t>
+  </si>
+  <si>
+    <t>Waste heat without additional burning</t>
+  </si>
+  <si>
+    <t>Geothermal</t>
+  </si>
+  <si>
+    <t>Heat from burning waste</t>
+  </si>
+  <si>
+    <t>HT</t>
+  </si>
+  <si>
+    <t>Waste heat Tata Steel</t>
+  </si>
+  <si>
+    <t>Waste heat from gas fired power plant</t>
+  </si>
+  <si>
+    <t>Waste heat from coal fired power plant</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1111/jiec.13047</t>
+  </si>
+  <si>
+    <t>Verhagen et al. 2020</t>
+  </si>
+  <si>
+    <t>kg CO2 per GJ</t>
+  </si>
+  <si>
+    <t>fuel according to Verhagen et al.</t>
+  </si>
 </sst>
 </file>
 
@@ -387,7 +511,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -422,6 +546,30 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -498,7 +646,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -528,11 +676,17 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="2" builtinId="5"/>
+    <cellStyle name="Per cent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -865,23 +1019,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA6EB78D-E0B7-4068-9041-25EE1114C448}">
   <dimension ref="A1:H25"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="35.86328125" customWidth="1"/>
-    <col min="2" max="2" width="23.73046875" customWidth="1"/>
-    <col min="3" max="3" width="19.1328125" customWidth="1"/>
-    <col min="4" max="4" width="17.265625" customWidth="1"/>
-    <col min="5" max="5" width="18.86328125" customWidth="1"/>
-    <col min="6" max="6" width="56.59765625" customWidth="1"/>
-    <col min="7" max="7" width="29.1328125" customWidth="1"/>
+    <col min="1" max="1" width="35.83203125" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" customWidth="1"/>
+    <col min="3" max="3" width="19.1640625" customWidth="1"/>
+    <col min="4" max="4" width="17.33203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="56.6640625" customWidth="1"/>
+    <col min="7" max="7" width="29.1640625" customWidth="1"/>
     <col min="8" max="8" width="29" customWidth="1"/>
-    <col min="9" max="9" width="15.59765625" customWidth="1"/>
-    <col min="10" max="10" width="11.86328125" customWidth="1"/>
-    <col min="11" max="11" width="12.3984375" customWidth="1"/>
-    <col min="12" max="12" width="12.1328125" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" customWidth="1"/>
+    <col min="10" max="10" width="11.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.33203125" customWidth="1"/>
+    <col min="12" max="12" width="12.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -904,7 +1058,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -927,7 +1081,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:8" ht="80" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -953,7 +1107,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -976,7 +1130,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -999,7 +1153,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -1022,7 +1176,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:8" ht="80" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -1048,7 +1202,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>24</v>
       </c>
@@ -1071,7 +1225,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>28</v>
       </c>
@@ -1094,7 +1248,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>31</v>
       </c>
@@ -1117,7 +1271,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>33</v>
       </c>
@@ -1140,7 +1294,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>35</v>
       </c>
@@ -1163,7 +1317,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>37</v>
       </c>
@@ -1186,7 +1340,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>39</v>
       </c>
@@ -1209,7 +1363,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>43</v>
       </c>
@@ -1232,7 +1386,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>45</v>
       </c>
@@ -1255,7 +1409,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>47</v>
       </c>
@@ -1278,7 +1432,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>49</v>
       </c>
@@ -1299,7 +1453,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>51</v>
       </c>
@@ -1320,7 +1474,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>53</v>
       </c>
@@ -1340,7 +1494,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>55</v>
       </c>
@@ -1363,7 +1517,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>59</v>
       </c>
@@ -1386,7 +1540,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>63</v>
       </c>
@@ -1406,7 +1560,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>65</v>
       </c>
@@ -1426,7 +1580,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>67</v>
       </c>
@@ -1492,13 +1646,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00BCDC15-0AA9-4C30-AC95-68925AD22B21}">
   <dimension ref="A1:S22"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="19" max="19" width="12.3984375" customWidth="1"/>
+    <col min="19" max="19" width="12.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
@@ -1557,7 +1711,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2" s="7" t="s">
         <v>6</v>
       </c>
@@ -1600,7 +1754,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
         <v>11</v>
       </c>
@@ -1653,7 +1807,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
         <v>15</v>
       </c>
@@ -1701,7 +1855,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
         <v>17</v>
       </c>
@@ -1744,7 +1898,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
         <v>19</v>
       </c>
@@ -1787,7 +1941,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
         <v>21</v>
       </c>
@@ -1830,7 +1984,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
         <v>24</v>
       </c>
@@ -1863,7 +2017,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
         <v>28</v>
       </c>
@@ -1901,7 +2055,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
         <v>31</v>
       </c>
@@ -1944,7 +2098,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
         <v>33</v>
       </c>
@@ -1982,7 +2136,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
         <v>35</v>
       </c>
@@ -2020,7 +2174,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
         <v>37</v>
       </c>
@@ -2058,7 +2212,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="s">
         <v>39</v>
       </c>
@@ -2106,7 +2260,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
         <v>43</v>
       </c>
@@ -2149,7 +2303,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
         <v>45</v>
       </c>
@@ -2182,7 +2336,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
         <v>47</v>
       </c>
@@ -2220,7 +2374,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
         <v>55</v>
       </c>
@@ -2263,7 +2417,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
         <v>59</v>
       </c>
@@ -2301,7 +2455,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A20" s="13" t="s">
         <v>67</v>
       </c>
@@ -2354,7 +2508,7 @@
         <v>20.399999999999999</v>
       </c>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A21" s="17" t="s">
         <v>79</v>
       </c>
@@ -2404,7 +2558,7 @@
         <v>0.99999999999999989</v>
       </c>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.2">
       <c r="B22" s="6"/>
       <c r="C22" s="6"/>
       <c r="D22" s="6"/>
@@ -2428,18 +2582,24 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBFA3CA6-DEFB-43EB-809E-2546365F8FF1}">
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="22" t="s">
         <v>82</v>
       </c>
       <c r="B1" s="22" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="C1" s="22" t="s">
+        <v>102</v>
+      </c>
+      <c r="D1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
         <v>68</v>
       </c>
@@ -2447,8 +2607,14 @@
         <f>'National average calculation'!D21</f>
         <v>0.42019607843137252</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="C2" s="27">
+        <v>32</v>
+      </c>
+      <c r="D2" s="26" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
         <v>70</v>
       </c>
@@ -2456,8 +2622,14 @@
         <f>'National average calculation'!F21</f>
         <v>0.20343137254901961</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="C3" s="27">
+        <v>26</v>
+      </c>
+      <c r="D3" s="26" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
         <v>77</v>
       </c>
@@ -2465,8 +2637,14 @@
         <f>'National average calculation'!H21</f>
         <v>4.4117647058823532E-2</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="C4" s="27">
+        <v>26</v>
+      </c>
+      <c r="D4" s="26" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
         <v>72</v>
       </c>
@@ -2474,8 +2652,14 @@
         <f>'National average calculation'!J21</f>
         <v>0.16058823529411767</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="C5" s="27">
+        <v>13</v>
+      </c>
+      <c r="D5" s="26" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
         <v>80</v>
       </c>
@@ -2483,8 +2667,14 @@
         <f>'National average calculation'!L21</f>
         <v>0.10245098039215686</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="C6" s="27">
+        <v>32</v>
+      </c>
+      <c r="D6" s="26" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
         <v>73</v>
       </c>
@@ -2492,8 +2682,14 @@
         <f>'National average calculation'!N21</f>
         <v>6.235294117647059E-2</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="C7" s="27">
+        <v>45</v>
+      </c>
+      <c r="D7" s="26" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
         <v>74</v>
       </c>
@@ -2501,8 +2697,14 @@
         <f>'National average calculation'!P21</f>
         <v>9.8039215686274508E-4</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="C8" s="28">
+        <v>13</v>
+      </c>
+      <c r="D8" s="26" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="9" t="s">
         <v>75</v>
       </c>
@@ -2510,8 +2712,195 @@
         <f>'National average calculation'!R21</f>
         <v>5.8823529411764705E-3</v>
       </c>
+      <c r="C9" s="27">
+        <v>13</v>
+      </c>
+      <c r="D9" s="26" t="s">
+        <v>91</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EAA1421F-687F-D44F-940A-15C91A3CE03D}">
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="20" x14ac:dyDescent="0.2">
+      <c r="B3" s="23" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="20" x14ac:dyDescent="0.2">
+      <c r="B4" s="23" t="s">
+        <v>84</v>
+      </c>
+      <c r="C4" s="23" t="s">
+        <v>85</v>
+      </c>
+      <c r="D4" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="E4" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="F4" s="23" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="20" x14ac:dyDescent="0.2">
+      <c r="B5" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="C5" s="24"/>
+      <c r="D5" s="24">
+        <v>192.8</v>
+      </c>
+      <c r="E5" s="24">
+        <v>1</v>
+      </c>
+      <c r="F5" s="24" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="20" x14ac:dyDescent="0.2">
+      <c r="B6" s="24" t="s">
+        <v>91</v>
+      </c>
+      <c r="C6" s="25">
+        <v>13000</v>
+      </c>
+      <c r="D6" s="24">
+        <v>46.8</v>
+      </c>
+      <c r="E6" s="24">
+        <v>0.24</v>
+      </c>
+      <c r="F6" s="24" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="20" x14ac:dyDescent="0.2">
+      <c r="B7" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="C7" s="25">
+        <v>8800</v>
+      </c>
+      <c r="D7" s="24">
+        <v>31.7</v>
+      </c>
+      <c r="E7" s="24">
+        <v>0.16</v>
+      </c>
+      <c r="F7" s="24" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="20" x14ac:dyDescent="0.2">
+      <c r="B8" s="24" t="s">
+        <v>94</v>
+      </c>
+      <c r="C8" s="25">
+        <v>25050</v>
+      </c>
+      <c r="D8" s="24">
+        <v>90.1</v>
+      </c>
+      <c r="E8" s="24">
+        <v>0.47</v>
+      </c>
+      <c r="F8" s="24" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="20" x14ac:dyDescent="0.2">
+      <c r="B9" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="C9" s="25">
+        <v>26000</v>
+      </c>
+      <c r="D9" s="24">
+        <v>93.6</v>
+      </c>
+      <c r="E9" s="24">
+        <v>0.49</v>
+      </c>
+      <c r="F9" s="24" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="20" x14ac:dyDescent="0.2">
+      <c r="B10" s="24" t="s">
+        <v>97</v>
+      </c>
+      <c r="C10" s="25">
+        <v>26000</v>
+      </c>
+      <c r="D10" s="24">
+        <v>93.6</v>
+      </c>
+      <c r="E10" s="24">
+        <v>0.49</v>
+      </c>
+      <c r="F10" s="24" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="20" x14ac:dyDescent="0.2">
+      <c r="B11" s="24" t="s">
+        <v>98</v>
+      </c>
+      <c r="C11" s="25">
+        <v>32000</v>
+      </c>
+      <c r="D11" s="24">
+        <v>115.2</v>
+      </c>
+      <c r="E11" s="24">
+        <v>0.6</v>
+      </c>
+      <c r="F11" s="24" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="20" x14ac:dyDescent="0.2">
+      <c r="B12" s="24" t="s">
+        <v>99</v>
+      </c>
+      <c r="C12" s="25">
+        <v>45000</v>
+      </c>
+      <c r="D12" s="24">
+        <v>162</v>
+      </c>
+      <c r="E12" s="24">
+        <v>0.84</v>
+      </c>
+      <c r="F12" s="24" t="s">
+        <v>96</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B1" r:id="rId1" xr:uid="{7D29EA95-3140-0645-9A1A-D9AA46759328}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>